<commit_message>
Arnold test set added. Prep work for 2024
</commit_message>
<xml_diff>
--- a/spread_sheets/out_2023.xlsx
+++ b/spread_sheets/out_2023.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="test_results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -978,7 +978,7 @@
         <v>-12.60208015119169</v>
       </c>
       <c r="C41" t="n">
-        <v>-6.593628519069306</v>
+        <v>-18.61053178331407</v>
       </c>
       <c r="D41" t="n">
         <v>1592</v>
@@ -992,7 +992,7 @@
         <v>-9.750983470890873</v>
       </c>
       <c r="C42" t="n">
-        <v>-3.742531838768492</v>
+        <v>-15.75943510301325</v>
       </c>
       <c r="D42" t="n">
         <v>160</v>
@@ -1006,7 +1006,7 @@
         <v>-8.05017020255594</v>
       </c>
       <c r="C43" t="n">
-        <v>-2.041718570433559</v>
+        <v>-14.05862183467832</v>
       </c>
       <c r="D43" t="n">
         <v>1592</v>
@@ -1020,7 +1020,7 @@
         <v>-4.600518422437361</v>
       </c>
       <c r="C44" t="n">
-        <v>1.407933209685019</v>
+        <v>-10.60897005455974</v>
       </c>
       <c r="D44" t="n">
         <v>160</v>
@@ -1034,7 +1034,7 @@
         <v>-6.750294033297521</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.7418424011751412</v>
+        <v>-12.7587456654199</v>
       </c>
       <c r="D45" t="n">
         <v>1592</v>
@@ -1048,7 +1048,7 @@
         <v>-5.25029403286581</v>
       </c>
       <c r="C46" t="n">
-        <v>0.7581575992565703</v>
+        <v>-11.25874566498819</v>
       </c>
       <c r="D46" t="n">
         <v>160</v>
@@ -1062,7 +1062,7 @@
         <v>-6.355740597707715</v>
       </c>
       <c r="C47" t="n">
-        <v>-0.3472889655853351</v>
+        <v>-12.3641922298301</v>
       </c>
       <c r="D47" t="n">
         <v>1592</v>
@@ -1076,7 +1076,7 @@
         <v>-3.305050141788612</v>
       </c>
       <c r="C48" t="n">
-        <v>2.703401490333768</v>
+        <v>-9.313501773910993</v>
       </c>
       <c r="D48" t="n">
         <v>160</v>
@@ -1090,7 +1090,7 @@
         <v>-7.750892538238574</v>
       </c>
       <c r="C49" t="n">
-        <v>-1.742440906116194</v>
+        <v>-13.75934417036095</v>
       </c>
       <c r="D49" t="n">
         <v>1592</v>
@@ -1104,7 +1104,7 @@
         <v>-5.551767161104948</v>
       </c>
       <c r="C50" t="n">
-        <v>0.4566844710174323</v>
+        <v>-11.56021879322733</v>
       </c>
       <c r="D50" t="n">
         <v>160</v>
@@ -1118,7 +1118,7 @@
         <v>11.49939796207811</v>
       </c>
       <c r="C51" t="n">
-        <v>17.50784959420049</v>
+        <v>5.490946329955726</v>
       </c>
       <c r="D51" t="n">
         <v>1592</v>
@@ -1132,7 +1132,7 @@
         <v>23.14981472295585</v>
       </c>
       <c r="C52" t="n">
-        <v>29.15826635507823</v>
+        <v>17.14136309083347</v>
       </c>
       <c r="D52" t="n">
         <v>160</v>
@@ -1146,7 +1146,7 @@
         <v>23.14820304039067</v>
       </c>
       <c r="C53" t="n">
-        <v>29.15665467251305</v>
+        <v>17.13975140826829</v>
       </c>
       <c r="D53" t="n">
         <v>1592</v>
@@ -1160,7 +1160,7 @@
         <v>-17.80121034156146</v>
       </c>
       <c r="C54" t="n">
-        <v>-11.79275870943908</v>
+        <v>-23.80966197368384</v>
       </c>
       <c r="D54" t="n">
         <v>160</v>

</xml_diff>